<commit_message>
feat: add fake demo data with progress values and milestone statuses
- Add currentValue for each priority objective:
  - Nutrition Security: 79.2% (baseline 78%, target 81.9%)
  - Anxiety/Stress: 45.8% (baseline 47%, target 44% - decrease goal)
  - CRC Screening: 76.3% (baseline 75.1%, target 78.8%)
- Update milestone statuses for demo:
  - 3.1-m1, 5.1-m1, 5.1-m2: complete
  - 3.1-m2, 5.1-m3, 33.0-m1, 33.0-m2: in_progress
  - 33.0-m3: not_started (starts later per timeline)
- Include update-demo-data.js script for reference

To revert to real data later, set currentValue to empty in Excel and
milestone statuses back to not_started, then run npm run data:build:sample

Co-authored-by: Dcrandell-OCDOH <Dcrandell-OCDOH@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/template/chip-sample.xlsx
+++ b/template/chip-sample.xlsx
@@ -401,10 +401,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B10"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -496,31 +492,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W4"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
-    <col min="11" max="11" width="19.83203125" customWidth="1"/>
-    <col min="12" max="12" width="24.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="14.83203125" customWidth="1"/>
-    <col min="15" max="15" width="17.83203125" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" customWidth="1"/>
-    <col min="17" max="17" width="15.83203125" customWidth="1"/>
-    <col min="18" max="18" width="14.83203125" customWidth="1"/>
-    <col min="19" max="19" width="16.83203125" customWidth="1"/>
-    <col min="20" max="20" width="14.83203125" customWidth="1"/>
-    <col min="21" max="21" width="22.83203125" customWidth="1"/>
-    <col min="22" max="22" width="24.83203125" customWidth="1"/>
-    <col min="23" max="23" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -648,8 +619,8 @@
       <c r="R2">
         <v>2030</v>
       </c>
-      <c r="S2" t="str">
-        <v/>
+      <c r="S2">
+        <v>79.2</v>
       </c>
       <c r="T2" t="str">
         <v>Orange County Community Health Survey, 2024</v>
@@ -719,8 +690,8 @@
       <c r="R3">
         <v>2030</v>
       </c>
-      <c r="S3" t="str">
-        <v/>
+      <c r="S3">
+        <v>45.8</v>
       </c>
       <c r="T3" t="str">
         <v>Orange County Community Health Survey, 2024</v>
@@ -790,8 +761,8 @@
       <c r="R4">
         <v>2030</v>
       </c>
-      <c r="S4" t="str">
-        <v/>
+      <c r="S4">
+        <v>76.3</v>
       </c>
       <c r="T4" t="str">
         <v>NYS Behavioral Risk Factor Surveillance Survey (BRFSS), 2024</v>
@@ -816,16 +787,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H9"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -876,7 +837,7 @@
         <v>Once</v>
       </c>
       <c r="H2" t="str">
-        <v>not_started</v>
+        <v>complete</v>
       </c>
     </row>
     <row r="3">
@@ -902,7 +863,7 @@
         <v>Quarterly</v>
       </c>
       <c r="H3" t="str">
-        <v>not_started</v>
+        <v>in_progress</v>
       </c>
     </row>
     <row r="4">
@@ -928,7 +889,7 @@
         <v>Once</v>
       </c>
       <c r="H4" t="str">
-        <v>not_started</v>
+        <v>complete</v>
       </c>
     </row>
     <row r="5">
@@ -954,7 +915,7 @@
         <v>Once</v>
       </c>
       <c r="H5" t="str">
-        <v>not_started</v>
+        <v>complete</v>
       </c>
     </row>
     <row r="6">
@@ -980,7 +941,7 @@
         <v>Quarterly</v>
       </c>
       <c r="H6" t="str">
-        <v>not_started</v>
+        <v>in_progress</v>
       </c>
     </row>
     <row r="7">
@@ -1006,7 +967,7 @@
         <v>Quarterly</v>
       </c>
       <c r="H7" t="str">
-        <v>not_started</v>
+        <v>in_progress</v>
       </c>
     </row>
     <row r="8">
@@ -1032,7 +993,7 @@
         <v>Quarterly</v>
       </c>
       <c r="H8" t="str">
-        <v>not_started</v>
+        <v>in_progress</v>
       </c>
     </row>
     <row r="9">
@@ -1071,15 +1032,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G42"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>